<commit_message>
working on ClimOO-SDC2 and revisions
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations/ClimOO Imports.xlsx
+++ b/ClimOO material/materials for implementations/ClimOO Imports.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D319E58E-9BE9-044E-9B73-2DA03BE03B5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C2023E7-A8FA-0249-B12E-DCC0F147E8AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42340" yWindow="2400" windowWidth="28800" windowHeight="16340" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
+    <workbookView xWindow="35900" yWindow="2780" windowWidth="28800" windowHeight="16340" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
   </bookViews>
   <sheets>
     <sheet name="Ontologies reused" sheetId="3" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="358">
   <si>
     <t>Agri-Food Experiment Ontology</t>
   </si>
@@ -1275,7 +1275,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1284,18 +1284,17 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1309,24 +1308,21 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1685,7 +1681,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2C20A25-ACC7-684D-AF97-19E64433B7DC}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
@@ -1695,16 +1691,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1712,10 +1708,10 @@
       <c r="A2" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="15" t="s">
         <v>63</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -1726,10 +1722,10 @@
       <c r="A3" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="15" t="s">
         <v>65</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -1740,10 +1736,10 @@
       <c r="A4" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="15" t="s">
         <v>68</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -1754,10 +1750,10 @@
       <c r="A5" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="15" t="s">
         <v>279</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -1768,7 +1764,7 @@
       <c r="A6" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="3" t="s">
         <v>283</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -1782,10 +1778,10 @@
       <c r="A7" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="15" t="s">
         <v>290</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -1796,7 +1792,7 @@
       <c r="A8" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="3" t="s">
         <v>56</v>
       </c>
       <c r="C8" s="3" t="s">
@@ -1810,7 +1806,7 @@
       <c r="A9" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="3" t="s">
         <v>55</v>
       </c>
       <c r="C9" s="3" t="s">
@@ -1824,7 +1820,7 @@
       <c r="A10" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="3" t="s">
         <v>285</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1838,7 +1834,7 @@
       <c r="A11" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="3" t="s">
         <v>48</v>
       </c>
       <c r="C11" s="3" t="s">
@@ -1852,10 +1848,10 @@
       <c r="A12" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="28" t="s">
         <v>243</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="16" t="s">
         <v>242</v>
       </c>
       <c r="D12" s="3" t="s">
@@ -1866,10 +1862,10 @@
       <c r="A13" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="17" t="s">
         <v>302</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -1883,13 +1879,13 @@
       <c r="A14" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="15" t="s">
         <v>350</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="3" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1897,13 +1893,13 @@
       <c r="A15" s="3" t="s">
         <v>348</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="15" t="s">
         <v>349</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="3" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1911,29 +1907,45 @@
       <c r="A16" s="3" t="s">
         <v>353</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="15" t="s">
         <v>351</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="3" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="3" t="s">
         <v>354</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="15" t="s">
         <v>355</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>357</v>
       </c>
+    </row>
+    <row r="18" spans="1:6" s="26" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1948,6 +1960,7 @@
     <hyperlink ref="C14" r:id="rId9" xr:uid="{C2421EE3-BB83-9D4A-9C8C-281BF85200BB}"/>
     <hyperlink ref="C16" r:id="rId10" xr:uid="{B689930A-191F-074E-A7A5-5BCB8D8B0D15}"/>
     <hyperlink ref="C17" r:id="rId11" xr:uid="{80B29E5F-3DC4-E041-8B61-178FD4F918FC}"/>
+    <hyperlink ref="C18" r:id="rId12" xr:uid="{7B51019E-C24F-DD42-B2F2-096D41B9C626}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -1959,1315 +1972,1274 @@
   <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="75.5" style="30" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" style="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="110.5" style="30" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" style="30"/>
-    <col min="5" max="5" width="21.83203125" style="30" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="10.83203125" style="30"/>
+    <col min="1" max="1" width="75.5" style="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" style="22" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="110.5" style="22" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" style="22"/>
+    <col min="5" max="5" width="21.83203125" style="22" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="10.83203125" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="29" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:5" s="26" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="14" t="s">
         <v>328</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="19" t="s">
         <v>299</v>
       </c>
-      <c r="E1" s="23"/>
-    </row>
-    <row r="2" spans="1:5" s="29" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="E1" s="20"/>
+    </row>
+    <row r="2" spans="1:5" s="26" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="24"/>
-      <c r="E2" s="5" t="s">
+      <c r="D2" s="21"/>
+      <c r="E2" s="4" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="11" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="11" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="8" t="s">
+    <row r="5" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-    </row>
-    <row r="6" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+    </row>
+    <row r="6" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-    </row>
-    <row r="7" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+    </row>
+    <row r="7" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="11" t="s">
         <v>252</v>
       </c>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-    </row>
-    <row r="8" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="25" t="s">
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+    </row>
+    <row r="8" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="22" t="s">
         <v>336</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="11" t="s">
         <v>250</v>
       </c>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-    </row>
-    <row r="9" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+    </row>
+    <row r="9" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="23" t="s">
         <v>270</v>
       </c>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-    </row>
-    <row r="10" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+    </row>
+    <row r="10" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="11" t="s">
         <v>248</v>
       </c>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-    </row>
-    <row r="11" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="8" t="s">
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+    </row>
+    <row r="11" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="11" t="s">
         <v>261</v>
       </c>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-    </row>
-    <row r="12" spans="1:5" s="29" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="9" t="s">
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+    </row>
+    <row r="12" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="11" t="s">
         <v>245</v>
       </c>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-    </row>
-    <row r="13" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="8" t="s">
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+    </row>
+    <row r="13" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="11" t="s">
         <v>251</v>
       </c>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-    </row>
-    <row r="14" spans="1:5" s="29" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+    </row>
+    <row r="14" spans="1:5" s="26" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-    </row>
-    <row r="15" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="8" t="s">
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+    </row>
+    <row r="15" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-    </row>
-    <row r="16" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="8" t="s">
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+    </row>
+    <row r="16" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-    </row>
-    <row r="17" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+    </row>
+    <row r="17" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-    </row>
-    <row r="18" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="8" t="s">
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+    </row>
+    <row r="18" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="11" t="s">
         <v>241</v>
       </c>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-    </row>
-    <row r="19" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="7" t="s">
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+    </row>
+    <row r="19" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-    </row>
-    <row r="20" spans="1:5" s="29" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="9" t="s">
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+    </row>
+    <row r="20" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A20" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="B20" s="25" t="s">
+      <c r="B20" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="11" t="s">
         <v>240</v>
       </c>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-    </row>
-    <row r="21" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="4" t="s">
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+    </row>
+    <row r="21" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-    </row>
-    <row r="22" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="25" t="s">
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+    </row>
+    <row r="22" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="11" t="s">
         <v>234</v>
       </c>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-    </row>
-    <row r="23" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="25" t="s">
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+    </row>
+    <row r="23" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="C23" s="26" t="s">
+      <c r="C23" s="23" t="s">
         <v>331</v>
       </c>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-    </row>
-    <row r="24" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="4" t="s">
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+    </row>
+    <row r="24" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="C24" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-    </row>
-    <row r="25" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="10" t="s">
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+    </row>
+    <row r="25" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="12" t="s">
+      <c r="C25" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-    </row>
-    <row r="26" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+    </row>
+    <row r="26" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="C26" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-    </row>
-    <row r="27" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="25" t="s">
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+    </row>
+    <row r="27" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="22" t="s">
         <v>335</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="C27" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25"/>
-    </row>
-    <row r="28" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="10" t="s">
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+    </row>
+    <row r="28" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-    </row>
-    <row r="29" spans="1:5" s="29" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="10" t="s">
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+    </row>
+    <row r="29" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A29" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="27" t="s">
+      <c r="C29" s="24" t="s">
         <v>217</v>
       </c>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-    </row>
-    <row r="30" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="28" t="s">
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+    </row>
+    <row r="30" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="25" t="s">
         <v>334</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="12" t="s">
+      <c r="C30" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
-    </row>
-    <row r="31" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="10" t="s">
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+    </row>
+    <row r="31" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="C31" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="D31" s="25"/>
-      <c r="E31" s="25"/>
-    </row>
-    <row r="32" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="25" t="s">
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+    </row>
+    <row r="32" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="22" t="s">
         <v>333</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C32" s="11" t="s">
         <v>173</v>
       </c>
-      <c r="D32" s="25"/>
-      <c r="E32" s="25"/>
-    </row>
-    <row r="33" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="4" t="s">
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+    </row>
+    <row r="33" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C33" s="12" t="s">
+      <c r="C33" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-    </row>
-    <row r="34" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+    </row>
+    <row r="34" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D34" s="25"/>
-      <c r="E34" s="25"/>
-    </row>
-    <row r="35" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="7" t="s">
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+    </row>
+    <row r="35" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="C35" s="11" t="s">
         <v>213</v>
       </c>
-      <c r="D35" s="25"/>
-      <c r="E35" s="25"/>
-    </row>
-    <row r="36" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="7" t="s">
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
+    </row>
+    <row r="36" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="C36" s="12" t="s">
+      <c r="C36" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="D36" s="25"/>
-      <c r="E36" s="25"/>
-    </row>
-    <row r="37" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="7" t="s">
+      <c r="D36" s="22"/>
+      <c r="E36" s="22"/>
+    </row>
+    <row r="37" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="C37" s="12" t="s">
+      <c r="C37" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="D37" s="25"/>
-      <c r="E37" s="25"/>
-    </row>
-    <row r="38" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="10" t="s">
+      <c r="D37" s="22"/>
+      <c r="E37" s="22"/>
+    </row>
+    <row r="38" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="D38" s="25"/>
-      <c r="E38" s="25"/>
-    </row>
-    <row r="39" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="7" t="s">
+      <c r="D38" s="22"/>
+      <c r="E38" s="22"/>
+    </row>
+    <row r="39" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="C39" s="26" t="s">
+      <c r="C39" s="23" t="s">
         <v>273</v>
       </c>
-      <c r="D39" s="25"/>
-      <c r="E39" s="25"/>
-    </row>
-    <row r="40" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="8" t="s">
+      <c r="D39" s="22"/>
+      <c r="E39" s="22"/>
+    </row>
+    <row r="40" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="C40" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="D40" s="25"/>
-      <c r="E40" s="25"/>
-    </row>
-    <row r="41" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="4" t="s">
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
+    </row>
+    <row r="41" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="C41" s="12" t="s">
+      <c r="C41" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="D41" s="25"/>
-      <c r="E41" s="25"/>
-    </row>
-    <row r="42" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="4" t="s">
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+    </row>
+    <row r="42" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="C42" s="12" t="s">
+      <c r="C42" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="D42" s="25"/>
-      <c r="E42" s="25"/>
-    </row>
-    <row r="43" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="4" t="s">
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+    </row>
+    <row r="43" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B43" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="D43" s="25"/>
-      <c r="E43" s="25"/>
-    </row>
-    <row r="44" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
+      <c r="D43" s="22"/>
+      <c r="E43" s="22"/>
+    </row>
+    <row r="44" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B44" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="C44" s="11" t="s">
+      <c r="C44" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="D44" s="25"/>
-      <c r="E44" s="25"/>
-    </row>
-    <row r="45" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="25" t="s">
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+    </row>
+    <row r="45" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="22" t="s">
         <v>184</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="C45" s="4" t="s">
+      <c r="C45" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="D45" s="25"/>
-      <c r="E45" s="25"/>
-    </row>
-    <row r="46" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="4" t="s">
+      <c r="D45" s="22"/>
+      <c r="E45" s="22"/>
+    </row>
+    <row r="46" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B46" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C46" s="12" t="s">
+      <c r="C46" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="D46" s="25"/>
-      <c r="E46" s="25"/>
-    </row>
-    <row r="47" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="7" t="s">
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+    </row>
+    <row r="47" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C47" s="12" t="s">
+      <c r="C47" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D47" s="25"/>
-      <c r="E47" s="25"/>
-    </row>
-    <row r="48" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="4" t="s">
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+    </row>
+    <row r="48" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="B48" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C48" s="12" t="s">
+      <c r="C48" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="D48" s="25"/>
-      <c r="E48" s="25"/>
-    </row>
-    <row r="49" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="4" t="s">
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+    </row>
+    <row r="49" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="B49" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="C49" s="12" t="s">
+      <c r="C49" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="D49" s="25"/>
-      <c r="E49" s="25"/>
-    </row>
-    <row r="50" spans="1:5" s="29" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A50" s="13" t="s">
+      <c r="D49" s="22"/>
+      <c r="E49" s="22"/>
+    </row>
+    <row r="50" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A50" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B50" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C50" s="12" t="s">
+      <c r="C50" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="D50" s="25"/>
-      <c r="E50" s="25"/>
-    </row>
-    <row r="51" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="4" t="s">
+      <c r="D50" s="22"/>
+      <c r="E50" s="22"/>
+    </row>
+    <row r="51" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C51" s="12" t="s">
+      <c r="C51" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="D51" s="25"/>
-      <c r="E51" s="25"/>
-    </row>
-    <row r="52" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="25" t="s">
+      <c r="D51" s="22"/>
+      <c r="E51" s="22"/>
+    </row>
+    <row r="52" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="22" t="s">
         <v>236</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="C52" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="D52" s="25"/>
-      <c r="E52" s="25"/>
-    </row>
-    <row r="53" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="4" t="s">
+      <c r="D52" s="22"/>
+      <c r="E52" s="22"/>
+    </row>
+    <row r="53" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="B53" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="C53" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="D53" s="25"/>
-      <c r="E53" s="25"/>
-    </row>
-    <row r="54" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="4" t="s">
+      <c r="D53" s="22"/>
+      <c r="E53" s="22"/>
+    </row>
+    <row r="54" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="B54" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C54" s="12" t="s">
+      <c r="C54" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D54" s="25"/>
-      <c r="E54" s="25"/>
-    </row>
-    <row r="55" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="4" t="s">
+      <c r="D54" s="22"/>
+      <c r="E54" s="22"/>
+    </row>
+    <row r="55" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C55" s="12" t="s">
+      <c r="C55" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="D55" s="25"/>
-      <c r="E55" s="25"/>
-    </row>
-    <row r="56" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="8" t="s">
+      <c r="D55" s="22"/>
+      <c r="E55" s="22"/>
+    </row>
+    <row r="56" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B56" s="8" t="s">
+      <c r="B56" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C56" s="12" t="s">
+      <c r="C56" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="D56" s="25"/>
-      <c r="E56" s="25"/>
-    </row>
-    <row r="57" spans="1:5" s="29" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A57" s="13" t="s">
+      <c r="D56" s="22"/>
+      <c r="E56" s="22"/>
+    </row>
+    <row r="57" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A57" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B57" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C57" s="12" t="s">
+      <c r="C57" s="11" t="s">
         <v>176</v>
       </c>
-      <c r="D57" s="25"/>
-      <c r="E57" s="25"/>
-    </row>
-    <row r="58" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="7" t="s">
+      <c r="D57" s="22"/>
+      <c r="E57" s="22"/>
+    </row>
+    <row r="58" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="B58" s="4" t="s">
+      <c r="B58" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="C58" s="12" t="s">
+      <c r="C58" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="D58" s="25"/>
-      <c r="E58" s="25"/>
-    </row>
-    <row r="59" spans="1:5" s="29" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A59" s="9" t="s">
+      <c r="D58" s="22"/>
+      <c r="E58" s="22"/>
+    </row>
+    <row r="59" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A59" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B59" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C59" s="4" t="s">
+      <c r="C59" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="D59" s="25"/>
-      <c r="E59" s="25"/>
-    </row>
-    <row r="60" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="25" t="s">
+      <c r="D59" s="22"/>
+      <c r="E59" s="22"/>
+    </row>
+    <row r="60" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B60" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="C60" s="12" t="s">
+      <c r="C60" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="D60" s="25"/>
-      <c r="E60" s="25"/>
-    </row>
-    <row r="61" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="4" t="s">
+      <c r="D60" s="22"/>
+      <c r="E60" s="22"/>
+    </row>
+    <row r="61" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B61" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C61" s="11" t="s">
+      <c r="C61" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="D61" s="25"/>
-      <c r="E61" s="25"/>
-    </row>
-    <row r="62" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="4" t="s">
+      <c r="D61" s="22"/>
+      <c r="E61" s="22"/>
+    </row>
+    <row r="62" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="B62" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="C62" s="12" t="s">
+      <c r="C62" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="D62" s="25"/>
-      <c r="E62" s="25"/>
-    </row>
-    <row r="63" spans="1:5" s="29" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="8" t="s">
+      <c r="D62" s="22"/>
+      <c r="E62" s="22"/>
+    </row>
+    <row r="63" spans="1:5" s="26" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B63" s="8" t="s">
+      <c r="B63" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C63" s="12" t="s">
+      <c r="C63" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="D63" s="25"/>
-      <c r="E63" s="25"/>
-    </row>
-    <row r="64" spans="1:5" s="29" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A64" s="10" t="s">
+      <c r="D63" s="22"/>
+      <c r="E63" s="22"/>
+    </row>
+    <row r="64" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A64" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B64" s="8" t="s">
+      <c r="B64" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C64" s="14" t="s">
+      <c r="C64" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="D64" s="25"/>
-      <c r="E64" s="25"/>
-    </row>
-    <row r="65" spans="1:5" s="29" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A65" s="9" t="s">
+      <c r="D64" s="22"/>
+      <c r="E64" s="22"/>
+    </row>
+    <row r="65" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A65" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="B65" s="4" t="s">
+      <c r="B65" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C65" s="12" t="s">
+      <c r="C65" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="D65" s="25"/>
-      <c r="E65" s="25"/>
-    </row>
-    <row r="66" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="4" t="s">
+      <c r="D65" s="22"/>
+      <c r="E65" s="22"/>
+    </row>
+    <row r="66" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B66" s="4" t="s">
+      <c r="B66" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="C66" s="12" t="s">
+      <c r="C66" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="D66" s="25"/>
-      <c r="E66" s="25"/>
-    </row>
-    <row r="67" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="4" t="s">
+      <c r="D66" s="22"/>
+      <c r="E66" s="22"/>
+    </row>
+    <row r="67" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B67" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C67" s="12" t="s">
+      <c r="C67" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="D67" s="25"/>
-      <c r="E67" s="25"/>
-    </row>
-    <row r="68" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="4" t="s">
+      <c r="D67" s="22"/>
+      <c r="E67" s="22"/>
+    </row>
+    <row r="68" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B68" s="4" t="s">
+      <c r="B68" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="C68" s="12" t="s">
+      <c r="C68" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="D68" s="25"/>
-      <c r="E68" s="25"/>
-    </row>
-    <row r="69" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="4" t="s">
+      <c r="D68" s="22"/>
+      <c r="E68" s="22"/>
+    </row>
+    <row r="69" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B69" s="4" t="s">
+      <c r="B69" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="C69" s="12" t="s">
+      <c r="C69" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="D69" s="25"/>
-      <c r="E69" s="25"/>
-    </row>
-    <row r="70" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="7" t="s">
+      <c r="D69" s="22"/>
+      <c r="E69" s="22"/>
+    </row>
+    <row r="70" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="B70" s="4" t="s">
+      <c r="B70" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C70" s="26" t="s">
+      <c r="C70" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="D70" s="25"/>
-      <c r="E70" s="25"/>
-    </row>
-    <row r="71" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="4" t="s">
+      <c r="D70" s="22"/>
+      <c r="E70" s="22"/>
+    </row>
+    <row r="71" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="B71" s="4" t="s">
+      <c r="B71" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="C71" s="12" t="s">
+      <c r="C71" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="D71" s="25"/>
-      <c r="E71" s="25"/>
-    </row>
-    <row r="72" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="7" t="s">
+      <c r="D71" s="22"/>
+      <c r="E71" s="22"/>
+    </row>
+    <row r="72" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="B72" s="4" t="s">
+      <c r="B72" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="C72" s="12" t="s">
+      <c r="C72" s="11" t="s">
         <v>223</v>
       </c>
-      <c r="D72" s="25"/>
-      <c r="E72" s="25"/>
-    </row>
-    <row r="73" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="7" t="s">
+      <c r="D72" s="22"/>
+      <c r="E72" s="22"/>
+    </row>
+    <row r="73" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="B73" s="4" t="s">
+      <c r="B73" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="C73" s="12" t="s">
+      <c r="C73" s="11" t="s">
         <v>221</v>
       </c>
-      <c r="D73" s="25"/>
-      <c r="E73" s="25"/>
-    </row>
-    <row r="74" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="7" t="s">
+      <c r="D73" s="22"/>
+      <c r="E73" s="22"/>
+    </row>
+    <row r="74" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="B74" s="4" t="s">
+      <c r="B74" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="C74" s="12" t="s">
+      <c r="C74" s="11" t="s">
         <v>220</v>
       </c>
-      <c r="D74" s="25"/>
-      <c r="E74" s="25"/>
-    </row>
-    <row r="75" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="8" t="s">
+      <c r="D74" s="22"/>
+      <c r="E74" s="22"/>
+    </row>
+    <row r="75" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B75" s="8" t="s">
+      <c r="B75" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C75" s="12" t="s">
+      <c r="C75" s="11" t="s">
         <v>254</v>
       </c>
-      <c r="D75" s="25"/>
-      <c r="E75" s="25"/>
-    </row>
-    <row r="76" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="25" t="s">
+      <c r="D75" s="22"/>
+      <c r="E75" s="22"/>
+    </row>
+    <row r="76" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="B76" s="4" t="s">
+      <c r="B76" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="C76" s="12" t="s">
+      <c r="C76" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="D76" s="25"/>
-      <c r="E76" s="25"/>
-    </row>
-    <row r="77" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="8" t="s">
+      <c r="D76" s="22"/>
+      <c r="E76" s="22"/>
+    </row>
+    <row r="77" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B77" s="8" t="s">
+      <c r="B77" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C77" s="12" t="s">
+      <c r="C77" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="D77" s="25"/>
-      <c r="E77" s="25"/>
-    </row>
-    <row r="78" spans="1:5" s="29" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="9" t="s">
+      <c r="D77" s="22"/>
+      <c r="E77" s="22"/>
+    </row>
+    <row r="78" spans="1:5" s="26" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="B78" s="4" t="s">
+      <c r="B78" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="C78" s="26" t="s">
+      <c r="C78" s="23" t="s">
         <v>344</v>
       </c>
-      <c r="D78" s="25"/>
-      <c r="E78" s="25"/>
-    </row>
-    <row r="79" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="4" t="s">
+      <c r="D78" s="22"/>
+      <c r="E78" s="22"/>
+    </row>
+    <row r="79" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B79" s="4"/>
-      <c r="C79" s="4" t="s">
+      <c r="B79" s="3"/>
+      <c r="C79" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="D79" s="25"/>
-      <c r="E79" s="25"/>
-    </row>
-    <row r="80" spans="1:5" s="29" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="10" t="s">
+      <c r="D79" s="22"/>
+      <c r="E79" s="22"/>
+    </row>
+    <row r="80" spans="1:5" s="26" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B80" s="8"/>
-      <c r="C80" s="8" t="s">
+      <c r="B80" s="7"/>
+      <c r="C80" s="7" t="s">
         <v>343</v>
       </c>
-      <c r="D80" s="25"/>
-      <c r="E80" s="25"/>
-    </row>
-    <row r="81" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="4" t="s">
+      <c r="D80" s="22"/>
+      <c r="E80" s="22"/>
+    </row>
+    <row r="81" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B81" s="11"/>
-      <c r="C81" s="4" t="s">
+      <c r="B81" s="10"/>
+      <c r="C81" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="D81" s="25"/>
-      <c r="E81" s="25"/>
+      <c r="D81" s="22"/>
+      <c r="E81" s="22"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A82" s="4" t="s">
+      <c r="A82" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B82" s="11"/>
-      <c r="C82" s="12" t="s">
+      <c r="B82" s="10"/>
+      <c r="C82" s="11" t="s">
         <v>229</v>
       </c>
-      <c r="D82" s="25"/>
-      <c r="E82" s="25"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A83" s="8" t="s">
+      <c r="A83" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B83" s="8"/>
-      <c r="C83" s="8" t="s">
+      <c r="B83" s="7"/>
+      <c r="C83" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="D83" s="25"/>
-      <c r="E83" s="25"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A84" s="10" t="s">
+      <c r="A84" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B84" s="8"/>
-      <c r="C84" s="8" t="s">
+      <c r="B84" s="7"/>
+      <c r="C84" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D84" s="25"/>
-      <c r="E84" s="25"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A85" s="7" t="s">
+      <c r="A85" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B85" s="11"/>
-      <c r="C85" s="12" t="s">
+      <c r="B85" s="10"/>
+      <c r="C85" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="D85" s="25" t="s">
+      <c r="D85" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="E85" s="25"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A86" s="25" t="s">
+      <c r="A86" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="B86" s="11"/>
-      <c r="C86" s="12" t="s">
+      <c r="B86" s="10"/>
+      <c r="C86" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="D86" s="25"/>
-      <c r="E86" s="25"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A87" s="4" t="s">
+      <c r="A87" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B87" s="11"/>
-      <c r="C87" s="12" t="s">
+      <c r="B87" s="10"/>
+      <c r="C87" s="11" t="s">
         <v>174</v>
       </c>
-      <c r="D87" s="25"/>
-      <c r="E87" s="25"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A88" s="4" t="s">
+      <c r="A88" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B88" s="11"/>
-      <c r="C88" s="12" t="s">
+      <c r="B88" s="10"/>
+      <c r="C88" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="D88" s="25"/>
-      <c r="E88" s="25"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A89" s="4" t="s">
+      <c r="A89" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B89" s="11"/>
-      <c r="C89" s="12" t="s">
+      <c r="B89" s="10"/>
+      <c r="C89" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="D89" s="25"/>
-      <c r="E89" s="25"/>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A90" s="4" t="s">
+      <c r="A90" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B90" s="11"/>
-      <c r="C90" s="12" t="s">
+      <c r="B90" s="10"/>
+      <c r="C90" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="D90" s="25"/>
-      <c r="E90" s="25"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A91" s="4" t="s">
+      <c r="A91" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="B91" s="4" t="s">
+      <c r="B91" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="C91" s="26" t="s">
+      <c r="C91" s="23" t="s">
         <v>304</v>
       </c>
-      <c r="D91" s="25"/>
-      <c r="E91" s="25"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A92" s="4" t="s">
+      <c r="A92" s="3" t="s">
         <v>307</v>
       </c>
-      <c r="B92" s="4" t="s">
+      <c r="B92" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="C92" s="26" t="s">
+      <c r="C92" s="23" t="s">
         <v>308</v>
       </c>
-      <c r="D92" s="25"/>
-      <c r="E92" s="25"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A93" s="4" t="s">
+      <c r="A93" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="B93" s="4" t="s">
+      <c r="B93" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="C93" s="26" t="s">
+      <c r="C93" s="23" t="s">
         <v>342</v>
       </c>
-      <c r="D93" s="25"/>
-      <c r="E93" s="25"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A94" s="4" t="s">
+      <c r="A94" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="B94" s="4" t="s">
+      <c r="B94" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="C94" s="4" t="s">
+      <c r="C94" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="D94" s="25"/>
-      <c r="E94" s="25"/>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A95" s="4" t="s">
+      <c r="A95" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="B95" s="4" t="s">
+      <c r="B95" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="C95" s="26" t="s">
+      <c r="C95" s="23" t="s">
         <v>316</v>
       </c>
-      <c r="D95" s="25"/>
-      <c r="E95" s="25"/>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A96" s="4" t="s">
+      <c r="A96" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="B96" s="4" t="s">
+      <c r="B96" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="C96" s="26" t="s">
+      <c r="C96" s="23" t="s">
         <v>341</v>
       </c>
-      <c r="D96" s="25"/>
-      <c r="E96" s="25"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A97" s="4" t="s">
+      <c r="A97" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="B97" s="4" t="s">
+      <c r="B97" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="C97" s="4" t="s">
+      <c r="C97" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="D97" s="25"/>
-      <c r="E97" s="25"/>
     </row>
     <row r="98" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A98" s="9" t="s">
+      <c r="A98" s="8" t="s">
         <v>324</v>
       </c>
-      <c r="B98" s="4" t="s">
+      <c r="B98" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="C98" s="26" t="s">
+      <c r="C98" s="23" t="s">
         <v>323</v>
       </c>
-      <c r="D98" s="25"/>
-      <c r="E98" s="25"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A99" s="4" t="s">
+      <c r="A99" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="B99" s="4" t="s">
+      <c r="B99" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="C99" s="26" t="s">
+      <c r="C99" s="23" t="s">
         <v>327</v>
       </c>
-      <c r="D99" s="25"/>
-      <c r="E99" s="25"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A100" s="4" t="s">
+      <c r="A100" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="B100" s="4"/>
-      <c r="C100" s="26" t="s">
+      <c r="B100" s="3"/>
+      <c r="C100" s="23" t="s">
         <v>330</v>
       </c>
-      <c r="D100" s="25"/>
-      <c r="E100" s="25"/>
     </row>
     <row r="101" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A101" s="9" t="s">
+      <c r="A101" s="8" t="s">
         <v>338</v>
       </c>
-      <c r="B101" s="4" t="s">
+      <c r="B101" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="C101" s="26" t="s">
+      <c r="C101" s="23" t="s">
         <v>339</v>
       </c>
-      <c r="D101" s="25"/>
-      <c r="E101" s="25"/>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A102" s="4" t="s">
+      <c r="A102" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="B102" s="4" t="s">
+      <c r="B102" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="C102" s="26" t="s">
+      <c r="C102" s="23" t="s">
         <v>340</v>
       </c>
-      <c r="D102" s="25"/>
-      <c r="E102" s="25"/>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="s">
@@ -3276,7 +3248,7 @@
       <c r="B103" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C103" s="16" t="s">
+      <c r="C103" s="15" t="s">
         <v>72</v>
       </c>
       <c r="D103" s="3" t="s">
@@ -3290,28 +3262,28 @@
       <c r="B104" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="C104" s="17" t="s">
+      <c r="C104" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="D104" s="31" t="s">
+      <c r="D104" s="27" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="105" spans="1:6" s="29" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A105" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="B105" s="6" t="s">
+      <c r="B105" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C105" s="16" t="s">
+      <c r="C105" s="15" t="s">
         <v>268</v>
       </c>
-      <c r="D105" s="31" t="s">
+      <c r="D105" s="27" t="s">
         <v>69</v>
       </c>
-      <c r="E105" s="30"/>
-      <c r="F105" s="30"/>
+      <c r="E105" s="22"/>
+      <c r="F105" s="22"/>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" s="3" t="s">

</xml_diff>

<commit_message>
revising materials and related locations, adding SDC2 development protocol, revising ClimOO-SDC2
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations/ClimOO Imports.xlsx
+++ b/ClimOO material/materials for implementations/ClimOO Imports.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C2023E7-A8FA-0249-B12E-DCC0F147E8AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ECE0C8A-92A7-7B44-8445-185DF8C68F92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35900" yWindow="2780" windowWidth="28800" windowHeight="16340" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16460" activeTab="1" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Ontologies reused" sheetId="3" r:id="rId1"/>
-    <sheet name="Potential ontologies to reuse" sheetId="2" r:id="rId2"/>
+    <sheet name="PlasticO imports" sheetId="3" r:id="rId1"/>
+    <sheet name="ClimOO-SDC2 imports" sheetId="4" r:id="rId2"/>
+    <sheet name="PICCO imports" sheetId="5" r:id="rId3"/>
+    <sheet name="PICCOmela imports" sheetId="6" r:id="rId4"/>
+    <sheet name="Potential ontologies to reuse" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -37,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="365">
   <si>
     <t>Agri-Food Experiment Ontology</t>
   </si>
@@ -234,9 +237,6 @@
     <t>Sustainability Core Ontology</t>
   </si>
   <si>
-    <t>https://github.com/gioUbbiali/Sustainability-Core-Ontology</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Yes </t>
   </si>
   <si>
@@ -1111,13 +1111,37 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>Plastics Ontology</t>
+  </si>
+  <si>
+    <t>PlasticO</t>
+  </si>
+  <si>
+    <t>https://w3id.org/sco/repo</t>
+  </si>
+  <si>
+    <t>https://w3id.org/climoo/repo</t>
+  </si>
+  <si>
+    <t>ClimOO-SDC2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plastics Interconnecting with Climate Change Ontology </t>
+  </si>
+  <si>
+    <t>PICCO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://oborel.github.io/ </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1159,6 +1183,14 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1275,7 +1307,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1325,6 +1357,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1681,7 +1717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2C20A25-ACC7-684D-AF97-19E64433B7DC}">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
@@ -1725,151 +1761,151 @@
       <c r="B3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="29" t="s">
+        <v>359</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>65</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C4" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>278</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>279</v>
-      </c>
       <c r="D5" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>56</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>55</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>48</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" s="17" t="s">
         <v>301</v>
       </c>
-      <c r="C13" s="17" t="s">
-        <v>302</v>
-      </c>
       <c r="D13" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G13" t="s">
         <v>39</v>
@@ -1877,75 +1913,59 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>348</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>349</v>
-      </c>
       <c r="D15" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>350</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>353</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>352</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>351</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
+      <c r="C17" s="15" t="s">
+        <v>354</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>354</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>355</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="26" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1960,7 +1980,6 @@
     <hyperlink ref="C14" r:id="rId9" xr:uid="{C2421EE3-BB83-9D4A-9C8C-281BF85200BB}"/>
     <hyperlink ref="C16" r:id="rId10" xr:uid="{B689930A-191F-074E-A7A5-5BCB8D8B0D15}"/>
     <hyperlink ref="C17" r:id="rId11" xr:uid="{80B29E5F-3DC4-E041-8B61-178FD4F918FC}"/>
-    <hyperlink ref="C18" r:id="rId12" xr:uid="{7B51019E-C24F-DD42-B2F2-096D41B9C626}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -1968,6 +1987,329 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D1D5A97-5CAC-5842-B2F3-5274D7CBD229}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="10.83203125" style="32"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>359</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="26" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>267</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>289</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>364</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>348</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{BB3E1D17-2000-D34C-96CC-DAA12C596EC5}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{41C997C5-A948-0043-94C2-4425CCEDE6F1}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{7B51019E-C24F-DD42-B2F2-096D41B9C626}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{093EBB4A-361C-064F-A8A9-1CC47902DD3F}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{6FF9D3D0-63B1-434F-A4BF-A7D96AAEBD50}"/>
+    <hyperlink ref="C8" r:id="rId6" xr:uid="{B2E5C9E1-6D7E-6546-8243-BCE0B3C2C6CD}"/>
+    <hyperlink ref="C7" r:id="rId7" xr:uid="{E0037802-D06E-EC48-82DA-3BDF4AD4F7FC}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D59BB61F-DDC7-4246-B02E-C3A747084667}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>359</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="30" t="s">
+        <v>357</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>358</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>360</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="30" t="s">
+        <v>361</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>360</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{841F03E5-34F9-C04C-B821-DDB46A6D6D97}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{37654986-9F62-4B4C-B457-A8D17DB9AF3A}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{39655C6F-B271-D742-995A-C9200CD1CCC6}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{41B118D0-4AEF-C347-8FFC-4F506B3758CA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C9C16B9-D49A-C445-B342-A6E392AFD49A}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>359</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="30" t="s">
+        <v>357</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>358</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>360</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="30" t="s">
+        <v>361</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>360</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="30" t="s">
+        <v>362</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>363</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>360</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{6A8E79EC-5016-254D-AF8C-0CFEB3E7F663}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{60E3FEA7-98C0-5C41-962B-891B865EF4BF}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{E84407DC-2B3B-8C48-B228-6D5DF0DCF610}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{A886AA46-1201-C049-BAE1-906C5A36465C}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{F9F60964-C464-A04E-B457-88318BF0EB28}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B475128C-F7EE-8540-83D5-7C0DBC4F277D}">
   <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1988,10 +2330,10 @@
         <v>61</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E1" s="20"/>
     </row>
@@ -2007,29 +2349,29 @@
       </c>
       <c r="D2" s="21"/>
       <c r="E2" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="C3" s="11" t="s">
         <v>258</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
@@ -2040,98 +2382,98 @@
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D5" s="22"/>
       <c r="E5" s="22"/>
     </row>
     <row r="6" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
     </row>
     <row r="7" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
     </row>
     <row r="8" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="22" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>249</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>250</v>
       </c>
       <c r="D8" s="22"/>
       <c r="E8" s="22"/>
     </row>
     <row r="9" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>50</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D9" s="22"/>
       <c r="E9" s="22"/>
     </row>
     <row r="10" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="11" t="s">
         <v>247</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>248</v>
       </c>
       <c r="D10" s="22"/>
       <c r="E10" s="22"/>
     </row>
     <row r="11" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D11" s="22"/>
       <c r="E11" s="22"/>
     </row>
     <row r="12" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>99</v>
-      </c>
       <c r="C12" s="11" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D12" s="22"/>
       <c r="E12" s="22"/>
@@ -2144,27 +2486,27 @@
         <v>10</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D13" s="22"/>
       <c r="E13" s="22"/>
     </row>
     <row r="14" spans="1:5" s="26" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D14" s="22"/>
       <c r="E14" s="22"/>
     </row>
     <row r="15" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>11</v>
@@ -2177,7 +2519,7 @@
     </row>
     <row r="16" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>6</v>
@@ -2190,13 +2532,13 @@
     </row>
     <row r="17" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>119</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>120</v>
       </c>
       <c r="D17" s="22"/>
       <c r="E17" s="22"/>
@@ -2209,85 +2551,85 @@
         <v>14</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D18" s="22"/>
       <c r="E18" s="22"/>
     </row>
     <row r="19" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D19" s="22"/>
       <c r="E19" s="22"/>
     </row>
     <row r="20" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="B20" s="22" t="s">
-        <v>101</v>
-      </c>
       <c r="C20" s="11" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
     </row>
     <row r="21" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C21" s="11" t="s">
         <v>231</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>232</v>
       </c>
       <c r="D21" s="22"/>
       <c r="E21" s="22"/>
     </row>
     <row r="22" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C22" s="11" t="s">
         <v>233</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>234</v>
       </c>
       <c r="D22" s="22"/>
       <c r="E22" s="22"/>
     </row>
     <row r="23" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>168</v>
-      </c>
       <c r="C23" s="23" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D23" s="22"/>
       <c r="E23" s="22"/>
     </row>
     <row r="24" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="C24" s="11" t="s">
         <v>135</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>136</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="22"/>
@@ -2300,40 +2642,40 @@
         <v>42</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D25" s="22"/>
       <c r="E25" s="22"/>
     </row>
     <row r="26" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D26" s="22"/>
       <c r="E26" s="22"/>
     </row>
     <row r="27" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="22" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="C27" s="11" t="s">
         <v>204</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>205</v>
       </c>
       <c r="D27" s="22"/>
       <c r="E27" s="22"/>
     </row>
     <row r="28" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>30</v>
@@ -2352,20 +2694,20 @@
         <v>17</v>
       </c>
       <c r="C29" s="24" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D29" s="22"/>
       <c r="E29" s="22"/>
     </row>
     <row r="30" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="25" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D30" s="22"/>
       <c r="E30" s="22"/>
@@ -2378,33 +2720,33 @@
         <v>19</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D31" s="22"/>
       <c r="E31" s="22"/>
     </row>
     <row r="32" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="22" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B32" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C32" s="11" t="s">
         <v>172</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>173</v>
       </c>
       <c r="D32" s="22"/>
       <c r="E32" s="22"/>
     </row>
     <row r="33" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D33" s="22"/>
       <c r="E33" s="22"/>
@@ -2424,39 +2766,39 @@
     </row>
     <row r="35" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B35" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C35" s="11" t="s">
         <v>212</v>
-      </c>
-      <c r="C35" s="11" t="s">
-        <v>213</v>
       </c>
       <c r="D35" s="22"/>
       <c r="E35" s="22"/>
     </row>
     <row r="36" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="B36" s="3" t="s">
-        <v>211</v>
-      </c>
       <c r="C36" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D36" s="22"/>
       <c r="E36" s="22"/>
     </row>
     <row r="37" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D37" s="22"/>
       <c r="E37" s="22"/>
@@ -2469,20 +2811,20 @@
         <v>21</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D38" s="22"/>
       <c r="E38" s="22"/>
     </row>
     <row r="39" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B39" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="C39" s="23" t="s">
         <v>272</v>
-      </c>
-      <c r="C39" s="23" t="s">
-        <v>273</v>
       </c>
       <c r="D39" s="22"/>
       <c r="E39" s="22"/>
@@ -2495,202 +2837,202 @@
         <v>23</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D40" s="22"/>
       <c r="E40" s="22"/>
     </row>
     <row r="41" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="C41" s="11" t="s">
         <v>195</v>
-      </c>
-      <c r="C41" s="11" t="s">
-        <v>196</v>
       </c>
       <c r="D41" s="22"/>
       <c r="E41" s="22"/>
     </row>
     <row r="42" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B42" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="C42" s="11" t="s">
         <v>193</v>
-      </c>
-      <c r="C42" s="11" t="s">
-        <v>194</v>
       </c>
       <c r="D42" s="22"/>
       <c r="E42" s="22"/>
     </row>
     <row r="43" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B43" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="C43" s="3" t="s">
         <v>191</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>192</v>
       </c>
       <c r="D43" s="22"/>
       <c r="E43" s="22"/>
     </row>
     <row r="44" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B44" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C44" s="10" t="s">
         <v>188</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>189</v>
       </c>
       <c r="D44" s="22"/>
       <c r="E44" s="22"/>
     </row>
     <row r="45" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="22" t="s">
+        <v>183</v>
+      </c>
+      <c r="B45" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="C45" s="3" t="s">
         <v>185</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>186</v>
       </c>
       <c r="D45" s="22"/>
       <c r="E45" s="22"/>
     </row>
     <row r="46" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B46" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B46" s="3" t="s">
-        <v>126</v>
-      </c>
       <c r="C46" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D46" s="22"/>
       <c r="E46" s="22"/>
     </row>
     <row r="47" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D47" s="22"/>
       <c r="E47" s="22"/>
     </row>
     <row r="48" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D48" s="22"/>
       <c r="E48" s="22"/>
     </row>
     <row r="49" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B49" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="C49" s="11" t="s">
         <v>182</v>
-      </c>
-      <c r="C49" s="11" t="s">
-        <v>183</v>
       </c>
       <c r="D49" s="22"/>
       <c r="E49" s="22"/>
     </row>
     <row r="50" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="B50" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="B50" s="3" t="s">
-        <v>105</v>
-      </c>
       <c r="C50" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D50" s="22"/>
       <c r="E50" s="22"/>
     </row>
     <row r="51" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B51" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C51" s="11" t="s">
         <v>146</v>
-      </c>
-      <c r="C51" s="11" t="s">
-        <v>147</v>
       </c>
       <c r="D51" s="22"/>
       <c r="E51" s="22"/>
     </row>
     <row r="52" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="22" t="s">
+        <v>235</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="C52" s="3" t="s">
         <v>236</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="C52" s="3" t="s">
-        <v>237</v>
       </c>
       <c r="D52" s="22"/>
       <c r="E52" s="22"/>
     </row>
     <row r="53" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B53" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C53" s="3" t="s">
         <v>129</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>130</v>
       </c>
       <c r="D53" s="22"/>
       <c r="E53" s="22"/>
     </row>
     <row r="54" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D54" s="22"/>
       <c r="E54" s="22"/>
     </row>
     <row r="55" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C55" s="11" t="s">
         <v>169</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="C55" s="11" t="s">
-        <v>170</v>
       </c>
       <c r="D55" s="22"/>
       <c r="E55" s="22"/>
@@ -2703,85 +3045,85 @@
         <v>33</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D56" s="22"/>
       <c r="E56" s="22"/>
     </row>
     <row r="57" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="B57" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="B57" s="3" t="s">
-        <v>113</v>
-      </c>
       <c r="C57" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D57" s="22"/>
       <c r="E57" s="22"/>
     </row>
     <row r="58" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="B58" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="B58" s="3" t="s">
-        <v>179</v>
-      </c>
       <c r="C58" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D58" s="22"/>
       <c r="E58" s="22"/>
     </row>
     <row r="59" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B59" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B59" s="3" t="s">
-        <v>107</v>
-      </c>
       <c r="C59" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D59" s="22"/>
       <c r="E59" s="22"/>
     </row>
     <row r="60" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="B60" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="B60" s="3" t="s">
+      <c r="C60" s="11" t="s">
         <v>154</v>
-      </c>
-      <c r="C60" s="11" t="s">
-        <v>155</v>
       </c>
       <c r="D60" s="22"/>
       <c r="E60" s="22"/>
     </row>
     <row r="61" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D61" s="22"/>
       <c r="E61" s="22"/>
     </row>
     <row r="62" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B62" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C62" s="11" t="s">
         <v>150</v>
-      </c>
-      <c r="C62" s="11" t="s">
-        <v>151</v>
       </c>
       <c r="D62" s="22"/>
       <c r="E62" s="22"/>
@@ -2794,7 +3136,7 @@
         <v>37</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D63" s="22"/>
       <c r="E63" s="22"/>
@@ -2807,137 +3149,137 @@
         <v>35</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D64" s="22"/>
       <c r="E64" s="22"/>
     </row>
     <row r="65" spans="1:5" s="26" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A65" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="B65" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="B65" s="3" t="s">
-        <v>109</v>
-      </c>
       <c r="C65" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D65" s="22"/>
       <c r="E65" s="22"/>
     </row>
     <row r="66" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B66" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B66" s="3" t="s">
+      <c r="C66" s="11" t="s">
         <v>140</v>
-      </c>
-      <c r="C66" s="11" t="s">
-        <v>141</v>
       </c>
       <c r="D66" s="22"/>
       <c r="E66" s="22"/>
     </row>
     <row r="67" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B67" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C67" s="11" t="s">
         <v>137</v>
-      </c>
-      <c r="C67" s="11" t="s">
-        <v>138</v>
       </c>
       <c r="D67" s="22"/>
       <c r="E67" s="22"/>
     </row>
     <row r="68" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B68" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C68" s="11" t="s">
         <v>142</v>
-      </c>
-      <c r="C68" s="11" t="s">
-        <v>143</v>
       </c>
       <c r="D68" s="22"/>
       <c r="E68" s="22"/>
     </row>
     <row r="69" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C69" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D69" s="22"/>
       <c r="E69" s="22"/>
     </row>
     <row r="70" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A70" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C70" s="23" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D70" s="22"/>
       <c r="E70" s="22"/>
     </row>
     <row r="71" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="B71" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="B71" s="3" t="s">
-        <v>228</v>
-      </c>
       <c r="C71" s="11" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D71" s="22"/>
       <c r="E71" s="22"/>
     </row>
     <row r="72" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A72" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D72" s="22"/>
       <c r="E72" s="22"/>
     </row>
     <row r="73" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C73" s="11" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D73" s="22"/>
       <c r="E73" s="22"/>
     </row>
     <row r="74" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A74" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="B74" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="B74" s="3" t="s">
+      <c r="C74" s="11" t="s">
         <v>219</v>
-      </c>
-      <c r="C74" s="11" t="s">
-        <v>220</v>
       </c>
       <c r="D74" s="22"/>
       <c r="E74" s="22"/>
@@ -2950,20 +3292,20 @@
         <v>5</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D75" s="22"/>
       <c r="E75" s="22"/>
     </row>
     <row r="76" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A76" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="B76" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="B76" s="3" t="s">
+      <c r="C76" s="11" t="s">
         <v>160</v>
-      </c>
-      <c r="C76" s="11" t="s">
-        <v>161</v>
       </c>
       <c r="D76" s="22"/>
       <c r="E76" s="22"/>
@@ -2976,20 +3318,20 @@
         <v>44</v>
       </c>
       <c r="C77" s="11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D77" s="22"/>
       <c r="E77" s="22"/>
     </row>
     <row r="78" spans="1:5" s="26" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B78" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B78" s="3" t="s">
-        <v>111</v>
-      </c>
       <c r="C78" s="23" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D78" s="22"/>
       <c r="E78" s="22"/>
@@ -3000,7 +3342,7 @@
       </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D79" s="22"/>
       <c r="E79" s="22"/>
@@ -3011,29 +3353,29 @@
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D80" s="22"/>
       <c r="E80" s="22"/>
     </row>
     <row r="81" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B81" s="10"/>
       <c r="C81" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D81" s="22"/>
       <c r="E81" s="22"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B82" s="10"/>
       <c r="C82" s="11" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
@@ -3042,7 +3384,7 @@
       </c>
       <c r="B83" s="7"/>
       <c r="C83" s="7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -3056,11 +3398,11 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B85" s="10"/>
       <c r="C85" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D85" s="22" t="s">
         <v>39</v>
@@ -3068,249 +3410,249 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" s="22" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B86" s="10"/>
       <c r="C86" s="11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B87" s="10"/>
       <c r="C87" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B88" s="10"/>
       <c r="C88" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B89" s="10"/>
       <c r="C89" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B90" s="10"/>
       <c r="C90" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B91" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="C91" s="23" t="s">
         <v>303</v>
-      </c>
-      <c r="C91" s="23" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C92" s="23" t="s">
         <v>307</v>
-      </c>
-      <c r="B92" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="C92" s="23" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="B93" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="B93" s="3" t="s">
-        <v>310</v>
-      </c>
       <c r="C93" s="23" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="C94" s="3" t="s">
         <v>312</v>
-      </c>
-      <c r="B94" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="C94" s="3" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="C95" s="23" t="s">
         <v>315</v>
-      </c>
-      <c r="B95" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="C95" s="23" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="B96" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="B96" s="3" t="s">
-        <v>318</v>
-      </c>
       <c r="C96" s="23" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="98" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A98" s="8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B98" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C98" s="23" t="s">
         <v>322</v>
-      </c>
-      <c r="C98" s="23" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="C99" s="23" t="s">
         <v>326</v>
-      </c>
-      <c r="B99" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="C99" s="23" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B100" s="3"/>
       <c r="C100" s="23" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="101" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A101" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="C101" s="23" t="s">
         <v>338</v>
-      </c>
-      <c r="B101" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="C101" s="23" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B102" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="B102" s="3" t="s">
-        <v>275</v>
-      </c>
       <c r="C102" s="23" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B103" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B103" s="3" t="s">
+      <c r="C103" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="C103" s="15" t="s">
-        <v>72</v>
-      </c>
       <c r="D103" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B104" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C104" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="C104" s="16" t="s">
-        <v>157</v>
-      </c>
       <c r="D104" s="27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="105" spans="1:6" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A105" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B105" s="5" t="s">
         <v>49</v>
       </c>
       <c r="C105" s="15" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D105" s="27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E105" s="22"/>
       <c r="F105" s="22"/>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B106" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="B106" s="3" t="s">
+      <c r="C106" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="C106" s="3" t="s">
-        <v>276</v>
-      </c>
       <c r="D106" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>